<commit_message>
feat(pnl): add EBITDA adjustments, Reported EBITDA, and Management Adjusted EBITDA calculation engine
</commit_message>
<xml_diff>
--- a/sample_pnl_data.xlsx
+++ b/sample_pnl_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,44 +444,76 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Marketing_Advertising</t>
+          <t>Gain_Loss_on_Sales_of_Assets</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Payroll_Salaries</t>
+          <t>Depreciation_Amortization</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Taxes_Interest</t>
+          <t>Interest_Expense</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Other_Income_Expenses</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Other_Non_Operating_Expenses</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Income_Taxes</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Total_Adjustments</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>125000</v>
+        <v>107</v>
       </c>
       <c r="B2" t="n">
-        <v>-8500</v>
+        <v>-7</v>
       </c>
       <c r="C2" t="n">
-        <v>48000</v>
+        <v>52.5</v>
       </c>
       <c r="D2" t="n">
-        <v>12500</v>
+        <v>13.5</v>
       </c>
       <c r="E2" t="n">
-        <v>18500</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
-        <v>6500</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>24000</v>
+        <v>20</v>
       </c>
       <c r="H2" t="n">
-        <v>4200</v>
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>